<commit_message>
tabela sobre o uso das ias adicionada e horario de termino adicionado
</commit_message>
<xml_diff>
--- a/relatorio/Relatorio_de_Testes_CineLume.xlsx
+++ b/relatorio/Relatorio_de_Testes_CineLume.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aluno\Documents\cinelume-qa\relatorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BE34A1-A0AD-446C-A553-B27EA9897F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BC2F3A-39A8-4738-90C4-ADB9C61685F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="24" windowWidth="11784" windowHeight="12216" tabRatio="500" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="11784" windowHeight="12216" tabRatio="500" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Instrucoes" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="772">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="794">
   <si>
     <t>Relatório de Testes — CineLume v1.0</t>
   </si>
@@ -2370,6 +2370,72 @@
   </si>
   <si>
     <t>Numa próxima oportunidade, traria a automação de testes de ponta a ponta para mais cedo no cronograma e criaria cenários de carga ainda mais agressivos para simular picos de acessos em dias de estreia.</t>
+  </si>
+  <si>
+    <t>Gemini</t>
+  </si>
+  <si>
+    <t>Quais são as melhores técnicas para criar casos de teste baseados em particionamento de equivalência e análise de valor limite para validação de e-mail?</t>
+  </si>
+  <si>
+    <t>Explicou os conceitos teóricos de divisão de classes válidas e inválidas para campos de texto.</t>
+  </si>
+  <si>
+    <t>A ideia de organizar as colunas e separar bem os cenários positivos dos negativos.</t>
+  </si>
+  <si>
+    <t>Mudei os exemplos genéricos da IA para baterem certo com as regras do CineLume.</t>
+  </si>
+  <si>
+    <t>não usei ia</t>
+  </si>
+  <si>
+    <t>Quais são os pontos principais que devo avaliar para testar a performance e a segurança básica de uma aplicação web local?</t>
+  </si>
+  <si>
+    <t>Destacou a importância de medir o tempo de resposta e olhar os dados no console.</t>
+  </si>
+  <si>
+    <t>Os critérios para preencher os testes de carga e desempenho.</t>
+  </si>
+  <si>
+    <t>Adaptei tudo para os testes reais que fiz no navegador a testar o sistema.</t>
+  </si>
+  <si>
+    <t>Podes me dar um exemplo simples de como funciona uma função de teste unitário em JavaScript para comparar valores?</t>
+  </si>
+  <si>
+    <t>Mostrou uma estrutura básica de validação de resultados esperados versus obtidos.</t>
+  </si>
+  <si>
+    <t>A lógica para montar a tabela de resultados no HTML.</t>
+  </si>
+  <si>
+    <t>Reescrevi e ajustei para chamar as funções reais do regras.js.</t>
+  </si>
+  <si>
+    <t>Como posso escrever um resumo executivo de um relatório de testes recomendando liberar o sistema, mas com ressalvas?</t>
+  </si>
+  <si>
+    <t>Deu dicas de como equilibrar os pontos positivos com os bugs encontrados.</t>
+  </si>
+  <si>
+    <t>A forma de organizar o texto de forma profissional.</t>
+  </si>
+  <si>
+    <t>Coloquei os bugs reais do nosso projeto (assentos e pagamentos) e a decisão final do CineLume.</t>
+  </si>
+  <si>
+    <t>Como posso verificar de forma simples se a correção de um bug num formulário não afetou outras partes do sistema?</t>
+  </si>
+  <si>
+    <t>Explicou o conceito de teste de regressão e sugeriu reexecutar os cenários afetados.</t>
+  </si>
+  <si>
+    <t>A ideia de focar os testes nas funções ao redor da correção.</t>
+  </si>
+  <si>
+    <t>Executei manualmente os testes no sistema para validar a correção do BUG-01 e garantir que tudo funcionava.</t>
   </si>
 </sst>
 </file>
@@ -2517,7 +2583,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -2567,6 +2633,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="47" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4081,82 +4150,150 @@
         <v>411</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="B5" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>773</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>775</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>776</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
+      <c r="B6" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>777</v>
+      </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="B7" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>778</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>779</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>780</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>781</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>777</v>
+      </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B9" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>782</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>783</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>784</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>790</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>791</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>792</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="B11" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>786</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>787</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>788</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>789</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4697,7 +4834,9 @@
       <c r="A11" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="8"/>
+      <c r="B11" s="25">
+        <v>46296.013429398146</v>
+      </c>
       <c r="C11" s="9" t="s">
         <v>60</v>
       </c>

</xml_diff>